<commit_message>
trade bus and 32 cases
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ZAF_grids_kan/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\VerveStacks_ZAF_grids_kan\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{979904E6-EF16-40D5-89B9-92C6506E9657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E16CEFA-EE87-41E1-B717-99E4E07FF732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28898" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc" sheetId="7" r:id="rId1"/>
@@ -2773,9 +2773,6 @@
     <t>Transformer: e_w92348290-400_ZAF → e_w92348290-765_ZAF</t>
   </si>
   <si>
-    <t>e_ZA11-400_ZAF,e_ZA40-400_ZAF,e_ZA41-400_ZAF,e_ZA44-400_ZAF,e_w120941269-400_ZAF,e_w169647963-400_ZAF,e_w169789536-400_ZAF,e_w182042518-400_ZAF,e_w219384657-400_ZAF,e_w219384657-765_ZAF,e_w545652232-400_ZAF,e_w62193952-400_ZAF,e_w62218063-400_ZAF,e_w836844162-400_ZAF,e_w90454383-400_ZAF</t>
-  </si>
-  <si>
     <t>pcg</t>
   </si>
   <si>
@@ -2786,6 +2783,9 @@
   </si>
   <si>
     <t>*NCAP_AFC</t>
+  </si>
+  <si>
+    <t>e_ZA11-400_ZAF</t>
   </si>
 </sst>
 </file>
@@ -4682,7 +4682,7 @@
       </c>
       <c r="L27" t="str">
         <f>$V$28</f>
-        <v>e_ZA11-400_ZAF,e_ZA40-400_ZAF,e_ZA41-400_ZAF,e_ZA44-400_ZAF,e_w120941269-400_ZAF,e_w169647963-400_ZAF,e_w169789536-400_ZAF,e_w182042518-400_ZAF,e_w219384657-400_ZAF,e_w219384657-765_ZAF,e_w545652232-400_ZAF,e_w62193952-400_ZAF,e_w62218063-400_ZAF,e_w836844162-400_ZAF,e_w90454383-400_ZAF</v>
+        <v>e_ZA11-400_ZAF</v>
       </c>
       <c r="P27">
         <v>0</v>
@@ -4704,7 +4704,7 @@
       </c>
       <c r="K28" t="str">
         <f>$V$28</f>
-        <v>e_ZA11-400_ZAF,e_ZA40-400_ZAF,e_ZA41-400_ZAF,e_ZA44-400_ZAF,e_w120941269-400_ZAF,e_w169647963-400_ZAF,e_w169789536-400_ZAF,e_w182042518-400_ZAF,e_w219384657-400_ZAF,e_w219384657-765_ZAF,e_w545652232-400_ZAF,e_w62193952-400_ZAF,e_w62218063-400_ZAF,e_w836844162-400_ZAF,e_w90454383-400_ZAF</v>
+        <v>e_ZA11-400_ZAF</v>
       </c>
       <c r="P28">
         <v>0</v>
@@ -4719,7 +4719,7 @@
         <v>50</v>
       </c>
       <c r="V28" s="147" t="s">
-        <v>881</v>
+        <v>885</v>
       </c>
     </row>
   </sheetData>
@@ -4874,7 +4874,7 @@
         <v>11</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>1</v>
@@ -4949,13 +4949,13 @@
         <v>14</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="J10" s="6" t="s">
         <v>62</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="L10" s="3" t="s">
         <v>49</v>
@@ -5003,13 +5003,13 @@
         <v>14</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>62</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="L11" s="6" t="s">
         <v>66</v>
@@ -5208,7 +5208,7 @@
         <v>60</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="L18" s="3" t="s">
         <v>49</v>
@@ -5243,7 +5243,7 @@
         <v>60</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="L19" t="s">
         <v>66</v>

</xml_diff>